<commit_message>
2nd feature of live host finding almost done
</commit_message>
<xml_diff>
--- a/reports/report.xlsx
+++ b/reports/report.xlsx
@@ -450,16 +450,16 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>48928</v>
+        <v>54655</v>
       </c>
       <c r="C2" t="n">
-        <v>48928</v>
+        <v>63</v>
       </c>
       <c r="D2" t="n">
-        <v>48928</v>
+        <v>63</v>
       </c>
       <c r="E2" t="n">
-        <v>48928</v>
+        <v>63</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
fixed the timeout issue
</commit_message>
<xml_diff>
--- a/reports/report.xlsx
+++ b/reports/report.xlsx
@@ -450,16 +450,16 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>54655</v>
+        <v>71290</v>
       </c>
       <c r="C2" t="n">
-        <v>63</v>
+        <v>50</v>
       </c>
       <c r="D2" t="n">
-        <v>63</v>
+        <v>50</v>
       </c>
       <c r="E2" t="n">
-        <v>63</v>
+        <v>50</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
security work in progress
</commit_message>
<xml_diff>
--- a/reports/report.xlsx
+++ b/reports/report.xlsx
@@ -446,20 +446,20 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>google.com</t>
+          <t>github.com</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>64197</v>
+        <v>41168</v>
       </c>
       <c r="C2" t="n">
-        <v>866</v>
+        <v>127</v>
       </c>
       <c r="D2" t="n">
-        <v>594</v>
+        <v>56</v>
       </c>
       <c r="E2" t="n">
-        <v>866</v>
+        <v>127</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
changed the output format
</commit_message>
<xml_diff>
--- a/reports/report.xlsx
+++ b/reports/report.xlsx
@@ -450,16 +450,16 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>41126</v>
+        <v>4</v>
       </c>
       <c r="C2" t="n">
-        <v>124</v>
+        <v>2</v>
       </c>
       <c r="D2" t="n">
-        <v>75</v>
+        <v>6</v>
       </c>
       <c r="E2" t="n">
-        <v>124</v>
+        <v>2</v>
       </c>
     </row>
   </sheetData>

</xml_diff>